<commit_message>
Scope stories to migration: drop field creation and update-set steps
- custom fields, choices and reference data belong to the implementation
  team; the field-creation and reference-data stories are replaced by one
  target readiness check (MIG-02) that confirms the load files match
- update-set steps removed from stories and docs
- stories renumbered MIG-01..MIG-15 with all cross-references updated
- docs 01/05/07/08/10 and decisions D11-D13 reworded as dependencies on
  the implementation team; transform-map spec marks pending custom fields
  "confirm exists (implementation team)"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/mapping/mapping_workbook.xlsx
+++ b/mapping/mapping_workbook.xlsx
@@ -562,7 +562,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="49" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>(a) new u_cost_center reference to cmn_cost_center (b) department</t>
+          <t>(a) implementation team provides u_cost_center (reference to cmn_cost_center) (b) map to department</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>(a) if Finance reports by cost center; else (b)</t>
+          <t>Ask the implementation team whether u_cost_center will exist; if not, load to department (if departments carry cost centers) or keep it in the description</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Finance + implementation team</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>(a) 7 custom fields on pm_project (and the intake ones on dmn_demand) (b) append to description (c) create a linked Completed demand holding intake dates</t>
+          <t>(a) implementation team provides the 7 fields on pm_project (b) keep them in the description block</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>(a) - these drive leadership and cycle-time reporting. Built into target_mapping as u_ fields</t>
+          <t>(a) if the implementation team agrees - these drive leadership and cycle-time reporting. The load files already carry the columns; they are dropped if the fields do not exist</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Nordic PMO</t>
+          <t>Nordic PMO + implementation team</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>(a) add u_risk_health to project_status (b) drop</t>
+          <t>(a) implementation team provides u_risk_health on project_status (b) drop</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>(a) - one field; keeps the 6-indicator status view</t>
+          <t>(a) if the implementation team agrees; otherwise the Risk RAG is dropped</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>PMO</t>
+          <t>PMO + implementation team</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -10338,7 +10338,7 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="47" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -10553,7 +10553,7 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -10600,7 +10600,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -11955,7 +11955,7 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr"/>
@@ -12002,7 +12002,7 @@
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -13392,7 +13392,7 @@
       <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr"/>
@@ -13439,7 +13439,7 @@
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr"/>
@@ -14836,7 +14836,7 @@
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr"/>
@@ -14883,7 +14883,7 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr"/>
@@ -16332,7 +16332,7 @@
       <c r="K113" s="2" t="inlineStr"/>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M113" s="2" t="inlineStr"/>
@@ -16379,7 +16379,7 @@
       <c r="K114" s="2" t="inlineStr"/>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M114" s="2" t="inlineStr"/>
@@ -17612,7 +17612,7 @@
       <c r="K137" s="2" t="inlineStr"/>
       <c r="L137" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M137" s="2" t="inlineStr"/>
@@ -17769,7 +17769,7 @@
       <c r="K140" s="2" t="inlineStr"/>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M140" s="2" t="inlineStr">
@@ -17824,7 +17824,7 @@
       <c r="K141" s="2" t="inlineStr"/>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M141" s="2" t="inlineStr">
@@ -17875,7 +17875,7 @@
       <c r="K142" s="2" t="inlineStr"/>
       <c r="L142" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M142" s="2" t="inlineStr">
@@ -17926,7 +17926,7 @@
       <c r="K143" s="2" t="inlineStr"/>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M143" s="2" t="inlineStr">
@@ -17977,7 +17977,7 @@
       <c r="K144" s="2" t="inlineStr"/>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M144" s="2" t="inlineStr">
@@ -18028,7 +18028,7 @@
       <c r="K145" s="2" t="inlineStr"/>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M145" s="2" t="inlineStr">
@@ -18079,7 +18079,7 @@
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M146" s="2" t="inlineStr">
@@ -18334,7 +18334,7 @@
       <c r="K151" s="2" t="inlineStr"/>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M151" s="2" t="inlineStr"/>
@@ -18381,7 +18381,7 @@
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M152" s="2" t="inlineStr"/>
@@ -19798,7 +19798,7 @@
       <c r="K179" s="2" t="inlineStr"/>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>PROPOSED - create before load</t>
+          <t>custom - confirm exists (implementation team)</t>
         </is>
       </c>
       <c r="M179" s="2" t="inlineStr">

</xml_diff>